<commit_message>
Add dismiss handler to FocusViewWindow and update ScanWindow initialization
</commit_message>
<xml_diff>
--- a/Sessions/2nd October session 13.xlsx
+++ b/Sessions/2nd October session 13.xlsx
@@ -512,8 +512,18 @@
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>[03:22:20]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>[03:18:47] Attended (Didn't do Exam &amp; Homework).
+[03:22:20] Canceled.
+[03:18:47] Attended (Didn't do Exam &amp; Homework).</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>excel_import</t>

</xml_diff>